<commit_message>
Record the post-deploy verification
All four round 4 defects that were fixed are now verified against the running
app, and the Kalambur AMK record is repaired. Zero duplicate item names remain
anywhere. R4-D4 stays open pending a decision.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KoaQ4eWvxjonvc68P5KHjA
</commit_message>
<xml_diff>
--- a/SKB_Rice_Mundy_QA_Round4.xlsx
+++ b/SKB_Rice_Mundy_QA_Round4.xlsx
@@ -11,10 +11,11 @@
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Round 4 results" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Defects" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="All rounds" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Reconciliation" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Still to do" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="Observations" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Post-deploy" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="All rounds" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Reconciliation" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Still to do" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Observations" sheetId="8" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="332">
   <si>
     <t xml:space="preserve">SKB Rice Mundy — QA Round 4 (full sweep)</t>
   </si>
@@ -484,6 +485,135 @@
     <t xml:space="preserve">Open — needs a client decision</t>
   </si>
   <si>
+    <t xml:space="preserve">After the deploy — what was verified on the live site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bundle index-WOZfADgy.js. Everything below was re-checked against the running app, not against the code. This tab supersedes the 'awaiting deploy' statuses on the Defects and All rounds tabs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Before</t>
+  </si>
+  <si>
+    <t xml:space="preserve">After</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cache headers on the live site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">index.html: max-age=3600, and the old bundle 404'd into index.html at status 200 → blank page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">index.html: no-cache, no-store, must-revalidate. /assets/**: public, max-age=31536000, immutable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rename the three duplicate item records</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Every item save failed with 'Item name is required.' — 7 attempts, 7 server-side errors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All three renamed: HMT Boiled (4,922), HMT Boiled - Carshed (774), HMT Boiled - Godown (1,038). The Carshed record's trailing space was trimmed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Item editing in general</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No item could be edited at all — MRP, bag size or category included</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Item editing works for the first time. This was the blocker on the whole round 3 objective</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Edit the Kalambur AMK supplier payment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Row: debit 6,000 AND credit 4,000. Statement 13,000. Header 1,000. Report 'paid 10,000'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Row: credit 6,000, balance 5,000. Header 5,000. Report: purchased 11,000 / paid 6,000 / payable 5,000. Tile 5,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Do the four sources agree?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Every one of them disagreed, and each was wrong differently</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All four agree, and agree on the correct figure of Rs 5,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Self-repair of the damaged record</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The corrupted row and the skewed stored balance both persisted through a reload</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Both healed on a single edit, with no data migration — the recompute working as designed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">e9e44d2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The hang I introduced, then fixed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The same edit sat on 'Saving...' indefinitely: no error, no toast, nothing written</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Completed in about 7 seconds</t>
+  </si>
+  <si>
+    <t xml:space="preserve">—</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delete the two stale Sona Raw test records</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Two zero-stock duplicates left over from round 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Both deleted. Only the real 260-bag record remains</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Duplicate item names anywhere in the app</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HMT Boiled x3, Sona Raw x3 — indistinguishable in every picker</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZERO duplicates. The purchase item picker lists 16 items, every one uniquely identifiable. The mis-billing risk is closed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inventory reconciliation after all the changes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18 items / 8,301 bags</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16 items / 8,307 bags, re-summed row by row and matching the header exactly. The two deleted records held no stock</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No control, and no deleteCategory in the source</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unchanged — still open, and still needs a decision on what happens to items in a deleted category</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OPEN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verified</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One thing I got wrong, and how</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The balance recompute I shipped in 9e8c5b6 ran its Firestore query from inside the transaction. A query issued there can block on the same stream the transaction holds, so the payment edit hung on 'Saving...' forever — no error, no toast, no console entry, nothing written. I hit it on my first attempt to repair Kalambur AMK. All eight of my tests passed while the feature was unusable, because they tested the arithmetic and never the mechanics. Fixed in e9e44d2 by reading the ledger once before the transaction opens, with two tests that pin the ordering specifically: moving the read back inside turns one red while the other nine stay green.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Defect history across all four rounds</t>
   </si>
   <si>
@@ -607,18 +737,15 @@
     <t xml:space="preserve">An item could not be renamed</t>
   </si>
   <si>
-    <t xml:space="preserve">AddItemModal set disabled on the Item Name field. Unlocked — and that is what exposed R4-D2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fixed, deployed; blocked by R4-D2</t>
+    <t xml:space="preserve">AddItemModal set disabled on the Item Name field. Unlocked — and that is what exposed R4-D2. All three renames are now done</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fixed, verified round 4 (post-deploy)</t>
   </si>
   <si>
     <t xml:space="preserve">name was never sent in the update payload</t>
   </si>
   <si>
-    <t xml:space="preserve">Fixed, awaiting deploy</t>
-  </si>
-  <si>
     <t xml:space="preserve">isSupplier branch removed; balance now recomputed from the rows</t>
   </si>
   <si>
@@ -634,6 +761,15 @@
     <t xml:space="preserve">No deleteCategory exists anywhere</t>
   </si>
   <si>
+    <t xml:space="preserve">D6-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Balance recompute hung the payment edit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">My own regression in 9e8c5b6: the ledger query ran inside the Firestore transaction and blocked. Read hoisted out in e9e44d2</t>
+  </si>
+  <si>
     <t xml:space="preserve">Counts</t>
   </si>
   <si>
@@ -845,9 +981,6 @@
   </si>
   <si>
     <t xml:space="preserve">Not defects. Recorded because each is a decision someone may want to make, or a trap for whoever tests this next.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">What</t>
   </si>
   <si>
     <t xml:space="preserve">'Last Updated' never moves for a sale</t>
@@ -1130,6 +1263,10 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1150,19 +1287,11 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1195,6 +1324,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2310,15 +2443,13 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="60"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2331,406 +2462,237 @@
         <v>153</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B4" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="C3" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="E3" s="6" t="s">
+      <c r="C4" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="F3" s="6" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
+      <c r="D4" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="B4" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="C4" s="19" t="s">
-        <v>134</v>
-      </c>
-      <c r="D4" s="9" t="s">
+      <c r="E4" s="6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="B5" s="15" t="s">
         <v>157</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="C5" s="9" t="s">
         <v>158</v>
       </c>
-      <c r="F4" s="20" t="s">
+      <c r="D5" s="9" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
+      <c r="E5" s="13" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="B6" s="15" t="s">
         <v>160</v>
       </c>
-      <c r="B5" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="C5" s="19" t="s">
-        <v>134</v>
-      </c>
-      <c r="D5" s="9" t="s">
+      <c r="C6" s="9" t="s">
         <v>161</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="D6" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="F5" s="20" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
-        <v>115</v>
-      </c>
-      <c r="B6" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="C6" s="19" t="s">
-        <v>134</v>
-      </c>
-      <c r="D6" s="9" t="s">
+      <c r="E6" s="13" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="B7" s="15" t="s">
         <v>163</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="C7" s="9" t="s">
         <v>164</v>
       </c>
-      <c r="F6" s="20" t="s">
+      <c r="D7" s="9" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
+      <c r="E7" s="13" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="B8" s="15" t="s">
         <v>166</v>
       </c>
-      <c r="B7" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" s="21" t="s">
-        <v>147</v>
-      </c>
-      <c r="D7" s="9" t="s">
+      <c r="C8" s="9" t="s">
         <v>167</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="D8" s="9" t="s">
         <v>168</v>
       </c>
-      <c r="F7" s="20" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
+      <c r="E8" s="13" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="B9" s="15" t="s">
         <v>169</v>
       </c>
-      <c r="B8" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="C8" s="21" t="s">
+      <c r="C9" s="9" t="s">
         <v>170</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D9" s="9" t="s">
         <v>171</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E9" s="13" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="B10" s="15" t="s">
         <v>172</v>
       </c>
-      <c r="F8" s="20" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
+      <c r="C10" s="9" t="s">
         <v>173</v>
       </c>
-      <c r="B9" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="C9" s="21" t="s">
-        <v>170</v>
-      </c>
-      <c r="D9" s="9" t="s">
+      <c r="D10" s="9" t="s">
         <v>174</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E10" s="13" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="12" t="s">
         <v>175</v>
       </c>
-      <c r="F9" s="20" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="s">
+      <c r="B11" s="15" t="s">
         <v>176</v>
       </c>
-      <c r="B10" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="C10" s="21" t="s">
-        <v>170</v>
-      </c>
-      <c r="D10" s="9" t="s">
+      <c r="C11" s="9" t="s">
         <v>177</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="D11" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="F10" s="20" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="s">
+      <c r="E11" s="13" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="12" t="s">
         <v>179</v>
       </c>
-      <c r="B11" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="C11" s="21" t="s">
-        <v>170</v>
-      </c>
-      <c r="D11" s="9" t="s">
+      <c r="B12" s="15" t="s">
         <v>180</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="C12" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="F11" s="20" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="s">
+      <c r="D12" s="9" t="s">
         <v>182</v>
       </c>
-      <c r="B12" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="C12" s="21" t="s">
-        <v>170</v>
-      </c>
-      <c r="D12" s="9" t="s">
+      <c r="E12" s="13" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="B13" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="E12" s="9" t="s">
+      <c r="C13" s="9" t="s">
         <v>184</v>
-      </c>
-      <c r="F12" s="20" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="B13" s="18" t="n">
-        <v>3</v>
-      </c>
-      <c r="C13" s="22" t="s">
-        <v>143</v>
       </c>
       <c r="D13" s="9" t="s">
         <v>185</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="E13" s="13" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="B14" s="15" t="s">
         <v>186</v>
       </c>
-      <c r="F13" s="20" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="B14" s="18" t="n">
-        <v>3</v>
-      </c>
-      <c r="C14" s="22" t="s">
-        <v>143</v>
+      <c r="C14" s="9" t="s">
+        <v>187</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="E14" s="9" t="s">
         <v>188</v>
       </c>
-      <c r="F14" s="20" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="B15" s="18" t="n">
-        <v>3</v>
-      </c>
-      <c r="C15" s="21" t="s">
-        <v>147</v>
+      <c r="E14" s="13" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="B15" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>189</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>189</v>
-      </c>
-      <c r="E15" s="9" t="s">
         <v>190</v>
       </c>
-      <c r="F15" s="20" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="s">
+      <c r="E15" s="14" t="s">
         <v>191</v>
       </c>
-      <c r="B16" s="18" t="n">
-        <v>3</v>
-      </c>
-      <c r="C16" s="22" t="s">
-        <v>143</v>
-      </c>
-      <c r="D16" s="9" t="s">
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="E16" s="9" t="s">
+      <c r="B17" s="4" t="str">
+        <f aca="false">CONCATENATE(COUNTIF(E5:E15,"PASS")," of ",COUNTA(E5:E15)," verified on the live site; ",COUNTIF(E5:E15,"OPEN")," still open")</f>
+        <v>10 of 11 verified on the live site; 1 still open</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="18" t="s">
         <v>193</v>
       </c>
-      <c r="F16" s="20" t="s">
+    </row>
+    <row r="20" customFormat="false" ht="75.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="17" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="B17" s="18" t="n">
-        <v>4</v>
-      </c>
-      <c r="C17" s="19" t="s">
-        <v>134</v>
-      </c>
-      <c r="D17" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="E17" s="9" t="s">
-        <v>195</v>
-      </c>
-      <c r="F17" s="23" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="B18" s="18" t="n">
-        <v>4</v>
-      </c>
-      <c r="C18" s="19" t="s">
-        <v>134</v>
-      </c>
-      <c r="D18" s="9" t="s">
-        <v>139</v>
-      </c>
-      <c r="E18" s="9" t="s">
-        <v>197</v>
-      </c>
-      <c r="F18" s="23" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="B19" s="18" t="n">
-        <v>4</v>
-      </c>
-      <c r="C19" s="22" t="s">
-        <v>143</v>
-      </c>
-      <c r="D19" s="9" t="s">
-        <v>198</v>
-      </c>
-      <c r="E19" s="9" t="s">
-        <v>199</v>
-      </c>
-      <c r="F19" s="23" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="B20" s="18" t="n">
-        <v>4</v>
-      </c>
-      <c r="C20" s="21" t="s">
-        <v>147</v>
-      </c>
-      <c r="D20" s="9" t="s">
-        <v>200</v>
-      </c>
-      <c r="E20" s="9" t="s">
-        <v>201</v>
-      </c>
-      <c r="F20" s="24" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
-        <v>202</v>
-      </c>
-      <c r="D22" s="4" t="str">
-        <f aca="false">CONCATENATE(COUNTA($A$4:$A$20)," defects tracked in total")</f>
-        <v>17 defects tracked in total</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D23" s="10" t="str">
-        <f aca="false">CONCATENATE(COUNTIF($F$4:$F$20,"Fixed, verified round 3")+COUNTIF($F$4:$F$20,"Fixed, verified round 4")," fixed and verified against the live app")</f>
-        <v>12 fixed and verified against the live app</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D24" s="10" t="str">
-        <f aca="false">CONCATENATE(COUNTIF($F$4:$F$20,"Fixed, awaiting deploy")," fixed but not yet deployed")</f>
-        <v>3 fixed but not yet deployed</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D25" s="10" t="str">
-        <f aca="false">CONCATENATE(COUNTIF($F$4:$F$20,"Open*")," still open")</f>
-        <v>1 still open</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D26" s="25" t="str">
-        <f aca="false">CONCATENATE(COUNTIF($F$4:$F$20,"Fixed, deployed*")," fixed and deployed, but blocked by a defect found this round (R5-01)")</f>
-        <v>1 fixed and deployed, but blocked by a defect found this round (R5-01)</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D27" s="26" t="str">
-        <f aca="false">CONCATENATE("Buckets add to ",COUNTIF($F$4:$F$21,"Fixed, verified round 3")+COUNTIF($F$4:$F$21,"Fixed, verified round 4")+COUNTIF($F$4:$F$21,"Fixed, awaiting deploy")+COUNTIF($F$4:$F$21,"Open*")+COUNTIF($F$4:$F$21,"Fixed, deployed*")," of ",COUNTA($A$4:$A$21)," tracked")</f>
-        <v>Buckets add to 17 of 17 tracked</v>
-      </c>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A20:E20"/>
+  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -2746,6 +2708,463 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:F28"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="22"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="7" t="s">
+        <v>199</v>
+      </c>
+      <c r="B4" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" s="20" t="s">
+        <v>134</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>200</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="F4" s="21" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="B5" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="20" t="s">
+        <v>134</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>204</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>205</v>
+      </c>
+      <c r="F5" s="21" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="B6" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="20" t="s">
+        <v>134</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>206</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="F6" s="21" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="B7" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="22" t="s">
+        <v>147</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="F7" s="21" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="B8" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" s="22" t="s">
+        <v>213</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>215</v>
+      </c>
+      <c r="F8" s="21" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="B9" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" s="22" t="s">
+        <v>213</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>218</v>
+      </c>
+      <c r="F9" s="21" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7" t="s">
+        <v>219</v>
+      </c>
+      <c r="B10" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C10" s="22" t="s">
+        <v>213</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>220</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="F10" s="21" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="B11" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="22" t="s">
+        <v>213</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>223</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>224</v>
+      </c>
+      <c r="F11" s="21" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="B12" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="22" t="s">
+        <v>213</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>226</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>227</v>
+      </c>
+      <c r="F12" s="21" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B13" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="C13" s="23" t="s">
+        <v>143</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>229</v>
+      </c>
+      <c r="F13" s="21" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="B14" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="C14" s="23" t="s">
+        <v>143</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>231</v>
+      </c>
+      <c r="F14" s="21" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="B15" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15" s="22" t="s">
+        <v>147</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>233</v>
+      </c>
+      <c r="F15" s="21" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="B16" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" s="23" t="s">
+        <v>143</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>235</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>236</v>
+      </c>
+      <c r="F16" s="21" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="B17" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C17" s="20" t="s">
+        <v>134</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="E17" s="9" t="s">
+        <v>238</v>
+      </c>
+      <c r="F17" s="21" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="B18" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C18" s="20" t="s">
+        <v>134</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>239</v>
+      </c>
+      <c r="F18" s="21" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="B19" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C19" s="23" t="s">
+        <v>143</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>240</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>241</v>
+      </c>
+      <c r="F19" s="21" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="B20" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C20" s="22" t="s">
+        <v>147</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>242</v>
+      </c>
+      <c r="E20" s="9" t="s">
+        <v>243</v>
+      </c>
+      <c r="F20" s="24" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="12" t="s">
+        <v>244</v>
+      </c>
+      <c r="B21" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C21" s="23" t="s">
+        <v>143</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>245</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>246</v>
+      </c>
+      <c r="F21" s="21" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="D23" s="4" t="str">
+        <f aca="false">CONCATENATE(COUNTA($A$4:$A$21)," defects tracked across all four rounds")</f>
+        <v>18 defects tracked across all four rounds</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="D24" s="10" t="str">
+        <f aca="false">CONCATENATE(COUNTIF($F$4:$F$21,"Fixed, verified round 3")," fixed and verified in round 3")</f>
+        <v>8 fixed and verified in round 3</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="D25" s="10" t="str">
+        <f aca="false">CONCATENATE(COUNTIF($F$4:$F$21,"Fixed, verified round 4")," fixed and verified during round 4")</f>
+        <v>4 fixed and verified during round 4</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="D26" s="10" t="str">
+        <f aca="false">CONCATENATE(COUNTIF($F$4:$F$21,"Fixed, verified round 4 (post-deploy)")," fixed and verified after the round 4 deploy")</f>
+        <v>5 fixed and verified after the round 4 deploy</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="D27" s="10" t="str">
+        <f aca="false">CONCATENATE(COUNTIF($F$4:$F$21,"Open*")," still open — R4-D4, which needs a client decision")</f>
+        <v>1 still open — R4-D4, which needs a client decision</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="D28" s="25" t="str">
+        <f aca="false">CONCATENATE("Buckets account for ",COUNTIF($F$4:$F$21,"Fixed, verified round 3")+COUNTIF($F$4:$F$21,"Fixed, verified round 4")+COUNTIF($F$4:$F$21,"Fixed, verified round 4 (post-deploy)")+COUNTIF($F$4:$F$21,"Open*")," of ",COUNTA($A$4:$A$21)," tracked")</f>
+        <v>Buckets account for 18 of 18 tracked</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:E26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -2757,39 +3176,39 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>203</v>
+        <v>248</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>204</v>
+        <v>249</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>205</v>
+        <v>250</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>206</v>
+        <v>251</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>207</v>
+        <v>252</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>208</v>
+        <v>253</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>209</v>
+        <v>254</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>210</v>
-      </c>
-      <c r="B5" s="27" t="n">
+        <v>255</v>
+      </c>
+      <c r="B5" s="26" t="n">
         <v>18</v>
       </c>
-      <c r="C5" s="27" t="n">
+      <c r="C5" s="26" t="n">
         <v>18</v>
       </c>
       <c r="D5" s="8" t="n">
@@ -2797,17 +3216,17 @@
         <v>0</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>211</v>
+        <v>256</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>212</v>
-      </c>
-      <c r="B6" s="27" t="n">
+        <v>257</v>
+      </c>
+      <c r="B6" s="26" t="n">
         <v>8301</v>
       </c>
-      <c r="C6" s="27" t="n">
+      <c r="C6" s="26" t="n">
         <v>8301</v>
       </c>
       <c r="D6" s="8" t="n">
@@ -2815,17 +3234,17 @@
         <v>0</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>211</v>
+        <v>256</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>213</v>
-      </c>
-      <c r="B7" s="27" t="n">
+        <v>258</v>
+      </c>
+      <c r="B7" s="26" t="n">
         <v>8301</v>
       </c>
-      <c r="C7" s="27" t="n">
+      <c r="C7" s="26" t="n">
         <v>8301</v>
       </c>
       <c r="D7" s="8" t="n">
@@ -2833,17 +3252,17 @@
         <v>0</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>214</v>
+        <v>259</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>215</v>
-      </c>
-      <c r="B8" s="27" t="n">
+        <v>260</v>
+      </c>
+      <c r="B8" s="26" t="n">
         <v>12209350</v>
       </c>
-      <c r="C8" s="27" t="n">
+      <c r="C8" s="26" t="n">
         <v>12209350</v>
       </c>
       <c r="D8" s="8" t="n">
@@ -2851,17 +3270,17 @@
         <v>0</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>216</v>
+        <v>261</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>217</v>
-      </c>
-      <c r="B9" s="27" t="n">
+        <v>262</v>
+      </c>
+      <c r="B9" s="26" t="n">
         <v>18</v>
       </c>
-      <c r="C9" s="27" t="n">
+      <c r="C9" s="26" t="n">
         <v>18</v>
       </c>
       <c r="D9" s="8" t="n">
@@ -2869,17 +3288,17 @@
         <v>0</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>218</v>
+        <v>263</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
-        <v>219</v>
-      </c>
-      <c r="B10" s="27" t="n">
+        <v>264</v>
+      </c>
+      <c r="B10" s="26" t="n">
         <v>8301</v>
       </c>
-      <c r="C10" s="27" t="n">
+      <c r="C10" s="26" t="n">
         <v>8301</v>
       </c>
       <c r="D10" s="8" t="n">
@@ -2887,17 +3306,17 @@
         <v>0</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>220</v>
+        <v>265</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>221</v>
-      </c>
-      <c r="B11" s="27" t="n">
+        <v>266</v>
+      </c>
+      <c r="B11" s="26" t="n">
         <v>14185975</v>
       </c>
-      <c r="C11" s="27" t="n">
+      <c r="C11" s="26" t="n">
         <v>14185975</v>
       </c>
       <c r="D11" s="8" t="n">
@@ -2905,17 +3324,17 @@
         <v>0</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>222</v>
+        <v>267</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>223</v>
-      </c>
-      <c r="B12" s="27" t="n">
+        <v>268</v>
+      </c>
+      <c r="B12" s="26" t="n">
         <v>16</v>
       </c>
-      <c r="C12" s="27" t="n">
+      <c r="C12" s="26" t="n">
         <v>16</v>
       </c>
       <c r="D12" s="8" t="n">
@@ -2923,17 +3342,17 @@
         <v>0</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>224</v>
+        <v>269</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>225</v>
-      </c>
-      <c r="B13" s="27" t="n">
+        <v>270</v>
+      </c>
+      <c r="B13" s="26" t="n">
         <v>20500</v>
       </c>
-      <c r="C13" s="27" t="n">
+      <c r="C13" s="26" t="n">
         <v>20500</v>
       </c>
       <c r="D13" s="8" t="n">
@@ -2941,31 +3360,31 @@
         <v>0</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>224</v>
+        <v>269</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="28" t="s">
-        <v>226</v>
-      </c>
-      <c r="B14" s="29"/>
-      <c r="C14" s="29"/>
-      <c r="D14" s="30" t="n">
+      <c r="A14" s="27" t="s">
+        <v>271</v>
+      </c>
+      <c r="B14" s="28"/>
+      <c r="C14" s="28"/>
+      <c r="D14" s="29" t="n">
         <f aca="false">SUM(D5:D13)</f>
         <v>0</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>227</v>
+        <v>272</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="31" t="s">
-        <v>228</v>
+      <c r="A17" s="30" t="s">
+        <v>273</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>229</v>
+        <v>274</v>
       </c>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
@@ -2974,101 +3393,101 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>230</v>
+        <v>275</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>231</v>
+        <v>276</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>232</v>
+        <v>277</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>233</v>
+        <v>278</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>234</v>
+        <v>279</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="s">
-        <v>235</v>
-      </c>
-      <c r="B21" s="32" t="n">
+        <v>280</v>
+      </c>
+      <c r="B21" s="31" t="n">
         <v>1000</v>
       </c>
-      <c r="C21" s="32" t="n">
+      <c r="C21" s="31" t="n">
         <v>5000</v>
       </c>
-      <c r="D21" s="33" t="n">
+      <c r="D21" s="32" t="n">
         <f aca="false">B21-C21</f>
         <v>-4000</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>236</v>
+        <v>281</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="9" t="s">
-        <v>237</v>
-      </c>
-      <c r="B22" s="32" t="n">
+        <v>282</v>
+      </c>
+      <c r="B22" s="31" t="n">
         <v>13000</v>
       </c>
-      <c r="C22" s="32" t="n">
+      <c r="C22" s="31" t="n">
         <v>5000</v>
       </c>
-      <c r="D22" s="33" t="n">
+      <c r="D22" s="32" t="n">
         <f aca="false">B22-C22</f>
         <v>8000</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>238</v>
+        <v>283</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="9" t="s">
-        <v>239</v>
-      </c>
-      <c r="B23" s="32" t="n">
+        <v>284</v>
+      </c>
+      <c r="B23" s="31" t="n">
         <v>10000</v>
       </c>
-      <c r="C23" s="32" t="n">
+      <c r="C23" s="31" t="n">
         <v>6000</v>
       </c>
-      <c r="D23" s="33" t="n">
+      <c r="D23" s="32" t="n">
         <f aca="false">B23-C23</f>
         <v>4000</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>240</v>
+        <v>285</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="9" t="s">
-        <v>241</v>
-      </c>
-      <c r="B24" s="32" t="n">
+        <v>286</v>
+      </c>
+      <c r="B24" s="31" t="n">
         <v>1000</v>
       </c>
-      <c r="C24" s="32" t="n">
+      <c r="C24" s="31" t="n">
         <v>5000</v>
       </c>
-      <c r="D24" s="33" t="n">
+      <c r="D24" s="32" t="n">
         <f aca="false">B24-C24</f>
         <v>-4000</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>242</v>
+        <v>287</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="34" t="s">
-        <v>243</v>
-      </c>
-      <c r="B26" s="34"/>
-      <c r="C26" s="34"/>
-      <c r="D26" s="34"/>
-      <c r="E26" s="34"/>
+      <c r="A26" s="33" t="s">
+        <v>288</v>
+      </c>
+      <c r="B26" s="33"/>
+      <c r="C26" s="33"/>
+      <c r="D26" s="33"/>
+      <c r="E26" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3085,7 +3504,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -3101,26 +3520,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>244</v>
+        <v>289</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>245</v>
+        <v>290</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>246</v>
+        <v>291</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>247</v>
+        <v>292</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>248</v>
+        <v>293</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>249</v>
+        <v>294</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3128,13 +3547,13 @@
         <v>1</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>250</v>
+        <v>295</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>251</v>
-      </c>
-      <c r="D4" s="23" t="s">
-        <v>252</v>
+        <v>296</v>
+      </c>
+      <c r="D4" s="34" t="s">
+        <v>297</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3142,13 +3561,13 @@
         <v>2</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>253</v>
+        <v>298</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>254</v>
-      </c>
-      <c r="D5" s="20" t="s">
-        <v>255</v>
+        <v>299</v>
+      </c>
+      <c r="D5" s="21" t="s">
+        <v>300</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3156,13 +3575,13 @@
         <v>3</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>256</v>
+        <v>301</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>257</v>
-      </c>
-      <c r="D6" s="20" t="s">
-        <v>255</v>
+        <v>302</v>
+      </c>
+      <c r="D6" s="21" t="s">
+        <v>300</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3170,13 +3589,13 @@
         <v>4</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>258</v>
+        <v>303</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>259</v>
-      </c>
-      <c r="D7" s="20" t="s">
-        <v>255</v>
+        <v>304</v>
+      </c>
+      <c r="D7" s="21" t="s">
+        <v>300</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3184,13 +3603,13 @@
         <v>5</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>260</v>
+        <v>305</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>261</v>
-      </c>
-      <c r="D8" s="23" t="s">
-        <v>262</v>
+        <v>306</v>
+      </c>
+      <c r="D8" s="34" t="s">
+        <v>307</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3198,13 +3617,13 @@
         <v>6</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>263</v>
+        <v>308</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>264</v>
+        <v>309</v>
       </c>
       <c r="D9" s="24" t="s">
-        <v>265</v>
+        <v>310</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3212,13 +3631,13 @@
         <v>7</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>266</v>
+        <v>311</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>267</v>
-      </c>
-      <c r="D10" s="23" t="s">
-        <v>268</v>
+        <v>312</v>
+      </c>
+      <c r="D10" s="34" t="s">
+        <v>313</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3226,13 +3645,13 @@
         <v>8</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>269</v>
+        <v>314</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>270</v>
+        <v>315</v>
       </c>
       <c r="D11" s="24" t="s">
-        <v>265</v>
+        <v>310</v>
       </c>
     </row>
   </sheetData>
@@ -3246,7 +3665,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -3261,23 +3680,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>271</v>
+        <v>316</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>272</v>
+        <v>317</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>246</v>
+        <v>291</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>273</v>
+        <v>154</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>248</v>
+        <v>293</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3285,10 +3704,10 @@
         <v>1</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>274</v>
+        <v>318</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>275</v>
+        <v>319</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3296,10 +3715,10 @@
         <v>2</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>276</v>
+        <v>320</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>277</v>
+        <v>321</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3307,10 +3726,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>278</v>
+        <v>322</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>279</v>
+        <v>323</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3318,10 +3737,10 @@
         <v>4</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>280</v>
+        <v>324</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>281</v>
+        <v>325</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3329,10 +3748,10 @@
         <v>5</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>282</v>
+        <v>326</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>283</v>
+        <v>327</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3340,10 +3759,10 @@
         <v>6</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>284</v>
+        <v>328</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>285</v>
+        <v>329</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3351,10 +3770,10 @@
         <v>7</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>286</v>
+        <v>330</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>287</v>
+        <v>331</v>
       </c>
     </row>
   </sheetData>

</xml_diff>